<commit_message>
WIP snapshot: Levels 1-4 lessons still in review by background agents (not final)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/01-foundations/01-excel-interface-navigation/1.1-excel-interface-navigation.xlsx
+++ b/01-foundations/01-excel-interface-navigation/1.1-excel-interface-navigation.xlsx
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Click cell A600, which is in an empty row below the data, and press Ctrl+→. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
+          <t>Use the Name Box to go to cell A600, which is in an empty row below the data, then press Ctrl+→. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -1224,7 +1224,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="51" customHeight="1">
+    <row r="12" ht="81" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
         <is>
           <t>7</t>
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B12" s="19" t="inlineStr">
         <is>
-          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl+Shift+↓ to select every date of birth. What is the date of birth of the oldest patient?</t>
+          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl+Shift+↓ to select every date of birth. What is the date of birth of the oldest patient? Type it as month/day/year, the way the status bar shows it. (If your computer uses day/month dates, type the month as a word instead, such as 15 Mar 1950.)</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl+F to find patient PT12376. What is that patient's phone number?</t>
+          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl+F (Mac: Control+F) to find patient PT12376. What is that patient's phone number?</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
@@ -38967,10 +38967,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="64" customHeight="1">
+    <row r="2" ht="79" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>The population-health team wants to use this patient list for a flu-shot outreach campaign. Before it goes out, the data steward asks you to check four facts. Set up first on the Patients sheet: if you froze panes earlier, choose View → Freeze Panes → Unfreeze Panes. Then press Ctrl+Home, click B2, and choose View → Freeze Panes → Freeze Panes so the headers and the PatientID column stay in view. Also turn on Minimum and Maximum in the status bar. You'll look everything up on the Patients sheet and type your answers on the Bonus sheet, and you won't need a single formula.</t>
+          <t>The population-health team is starting a blood-pressure outreach program and will build its mailing list from this patient index. Before the letters go out, the data steward asks you to check four facts. Set up the Patients sheet first: if you froze panes earlier, choose View → Freeze Panes → Unfreeze Panes. Then press Ctrl+Home (Mac: Control+Home), click B2, and choose View → Freeze Panes → Freeze Panes so the headers and the PatientID column stay in view. Also turn on Minimum and Maximum in the status bar. You'll look everything up on the Patients sheet and type your answers on the Bonus sheet, without a single formula.</t>
         </is>
       </c>
     </row>
@@ -39022,7 +39022,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Use Go To (F5 or Ctrl+G, Mac: Control+G) to select M2:M501. A blank PCPProviderID means the patient has no primary care provider on file. How many of the 500 patients have no PCP?</t>
+          <t>Each outreach letter is signed by the patient's primary care provider (PCP), and a blank PCPProviderID means no PCP is on file. Use Go To (F5 or Ctrl+G, Mac: Control+G) to select M2:M501. How many of the 500 patients have no PCP?</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -39036,7 +39036,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="66" customHeight="1">
+    <row r="7" ht="81" customHeight="1">
       <c r="A7" s="18" t="inlineStr">
         <is>
           <t>B2</t>
@@ -39044,7 +39044,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl+F (Mac: Control+F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN (hypertension). How many patients have HTN anywhere in their ChronicConditions list?</t>
+          <t>The program targets every patient with hypertension, coded HTN. Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl+F (Mac: Control+F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN. How many patients have HTN anywhere in their ChronicConditions list?</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -39058,7 +39058,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1">
+    <row r="8" ht="51" customHeight="1">
       <c r="A8" s="18" t="inlineStr">
         <is>
           <t>B3</t>
@@ -39066,7 +39066,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Now turn ON Match entire cell contents and Find All for HTN again. How many patients have hypertension as their ONLY recorded chronic condition?</t>
+          <t>Patients whose only condition is hypertension will get a shorter letter. Turn ON Match entire cell contents and Find All for HTN again. How many patients have hypertension as their ONLY recorded chronic condition?</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
@@ -39080,7 +39080,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="51" customHeight="1">
+    <row r="9" ht="66" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>B4</t>
@@ -39088,7 +39088,7 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>Which patient is the heaviest? Select O2:O501, read Maximum on the status bar, then use Find to locate that weight and read the PatientID in the frozen column A. Type the PatientID.</t>
+          <t>Finally, the steward wants to confirm that the largest weight on file is real and not a typo. Which patient is the heaviest? Select O2:O501, read Maximum on the status bar, then use Find to locate that weight and read the PatientID in the frozen column A. Type the PatientID.</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
@@ -39258,7 +39258,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Click cell A600, which is in an empty row below the data, and press Ctrl+→. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
+          <t>Use the Name Box to go to cell A600, which is in an empty row below the data, then press Ctrl+→. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
         </is>
       </c>
       <c r="C7" s="31" t="inlineStr">
@@ -39270,7 +39270,7 @@
         <is>
           <t>1. Type A600 in the Name Box and press Enter.
 2. Press Ctrl+→. The Name Box shows XFD600.
-3. Press Ctrl+← (or Ctrl+Home) to come back.</t>
+3. Press Ctrl+← to come back to column A.</t>
         </is>
       </c>
       <c r="E7" cm="1" s="33">
@@ -39381,7 +39381,7 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl+Shift+↓ to select every date of birth. What is the date of birth of the oldest patient?</t>
+          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl+Shift+↓ to select every date of birth. What is the date of birth of the oldest patient? Type it as month/day/year, the way the status bar shows it. (If your computer uses day/month dates, type the month as a word instead, such as 15 Mar 1950.)</t>
         </is>
       </c>
       <c r="C11" s="36" t="n">
@@ -39443,7 +39443,7 @@
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl+F to find patient PT12376. What is that patient's phone number?</t>
+          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl+F (Mac: Control+F) to find patient PT12376. What is that patient's phone number?</t>
         </is>
       </c>
       <c r="C13" s="31" t="inlineStr">
@@ -39639,7 +39639,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="81" customHeight="1">
+    <row r="5" ht="111" customHeight="1">
       <c r="A5" s="18" t="inlineStr">
         <is>
           <t>B1</t>
@@ -39647,7 +39647,7 @@
       </c>
       <c r="B5" s="19" t="inlineStr">
         <is>
-          <t>Use Go To (F5 or Ctrl+G, Mac: Control+G) to select M2:M501. A blank PCPProviderID means the patient has no primary care provider on file. How many of the 500 patients have no PCP?</t>
+          <t>Each outreach letter is signed by the patient's primary care provider (PCP), and a blank PCPProviderID means no PCP is on file. Use Go To (F5 or Ctrl+G, Mac: Control+G) to select M2:M501. How many of the 500 patients have no PCP?</t>
         </is>
       </c>
       <c r="C5" s="31" t="n">
@@ -39666,11 +39666,11 @@
       </c>
       <c r="F5" s="19" t="inlineStr">
         <is>
-          <t>Count only counts non-empty cells, so it tells you how many patients do have a PCP (469). The range M2:M501 covers rows 2 to 501, which is 500 cells, so 500 − 469 leaves 31 blanks. (If you select by dragging instead, the Name Box shows the size of the selection while you drag, such as 500R x 1C.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="96" customHeight="1">
+          <t>Count only counts non-empty cells, so it tells you how many patients do have a PCP (469). The range M2:M501 covers rows 2 to 501, which is 500 cells, so 500 − 469 leaves 31 blanks. Any of those patients who have hypertension need a PCP assigned before a letter can go out. (If you select by dragging instead, the Name Box shows the size of the selection while you drag, such as 500R x 1C.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="111" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
         <is>
           <t>B2</t>
@@ -39678,7 +39678,7 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl+F (Mac: Control+F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN (hypertension). How many patients have HTN anywhere in their ChronicConditions list?</t>
+          <t>The program targets every patient with hypertension, coded HTN. Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl+F (Mac: Control+F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN. How many patients have HTN anywhere in their ChronicConditions list?</t>
         </is>
       </c>
       <c r="C6" s="31" t="n">
@@ -39709,7 +39709,7 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>Now turn ON Match entire cell contents and Find All for HTN again. How many patients have hypertension as their ONLY recorded chronic condition?</t>
+          <t>Patients whose only condition is hypertension will get a shorter letter. Turn ON Match entire cell contents and Find All for HTN again. How many patients have hypertension as their ONLY recorded chronic condition?</t>
         </is>
       </c>
       <c r="C7" s="31" t="n">
@@ -39740,7 +39740,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>Which patient is the heaviest? Select O2:O501, read Maximum on the status bar, then use Find to locate that weight and read the PatientID in the frozen column A. Type the PatientID.</t>
+          <t>Finally, the steward wants to confirm that the largest weight on file is real and not a typo. Which patient is the heaviest? Select O2:O501, read Maximum on the status bar, then use Find to locate that weight and read the PatientID in the frozen column A. Type the PatientID.</t>
         </is>
       </c>
       <c r="C8" s="31" t="inlineStr">

</xml_diff>

<commit_message>
Course-wide consistency review fixes; curriculum is the source of truth for lesson level/time/objectives
- Fix cross-lesson contradictions, stale cross-references and version/shortcut drift found by the review
- Realistic lesson time estimates; README quote lines and objectives now synced from curriculum.py at build
- Start Here lists the Practice and Bonus sheets; data README gains common metric definitions
- Authoring guide: course-wide style conventions (Mac keys, menu paths, callouts, subsection numbering)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/01-foundations/01-excel-interface-navigation/1.1-excel-interface-navigation.xlsx
+++ b/01-foundations/01-excel-interface-navigation/1.1-excel-interface-navigation.xlsx
@@ -703,7 +703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:C31"/>
+  <dimension ref="B2:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -728,7 +728,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Beginner  ·  about 30 minutes  ·  Bluestone Health System (fictional)</t>
+          <t>Beginner  ·  about 70 minutes  ·  Bluestone Health System (fictional)</t>
         </is>
       </c>
     </row>
@@ -947,46 +947,70 @@
     <row r="28" ht="18" customHeight="1">
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Patients</t>
+          <t>Practice</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Data: 500 rows, in the Excel Table 'tblPatients'</t>
+          <t>12 practice tasks, each with a Check cell.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="B29" s="8" t="inlineStr">
         <is>
+          <t>Patients</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Data: 500 rows, in the Excel Table 'tblPatients'</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="B30" s="8" t="inlineStr">
+        <is>
           <t>Payers</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C30" s="7" t="inlineStr">
         <is>
           <t>Data: 8 rows, in the Excel Table 'tblPayers'</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="33" customHeight="1">
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>About the data</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>500 registered patients from the Bluestone Health System patient index (every 8th record), plus a small payer list that starts out hidden.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="B31" s="8" t="inlineStr">
         <is>
+          <t>Bonus</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>The bonus challenge (4 parts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="33" customHeight="1">
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>About the data</t>
+        </is>
+      </c>
+      <c r="C32" s="7" t="inlineStr">
+        <is>
+          <t>500 registered patients from the Bluestone Health System patient index (every 8th record), plus a small payer list that starts out hidden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="B33" s="8" t="inlineStr">
+        <is>
           <t>Disclaimer</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>All people, places, and numbers are synthetic and fictional. Not clinical guidance.</t>
         </is>

</xml_diff>

<commit_message>
Final polish: course-wide style conventions in every lesson, accurate Start Here sheet lists
- Every lesson: shortcut/Mac-key notation, Settings paths, bold menu paths, callout labels,
  subsection numbering, closing shortcuts/version reference section, version labels
- Start Here lists every visible sheet in tab order; sheet_notes can override data-sheet text
- Leftover review items (Find shortcuts, bonus-only sheet order, VBE wording, snippet placement)
- All 30 lessons rebuilt: verification PASS, no warnings

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/01-foundations/01-excel-interface-navigation/1.1-excel-interface-navigation.xlsx
+++ b/01-foundations/01-excel-interface-navigation/1.1-excel-interface-navigation.xlsx
@@ -820,7 +820,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
+    <row r="15" ht="33" customHeight="1">
       <c r="B15" s="8" t="inlineStr">
         <is>
           <t>2. Practice</t>
@@ -828,7 +828,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Go to the 'Practice' sheet. Type a formula or value into each yellow cell.</t>
+          <t>Go to the 'Practice' sheet. Each answer is something you read off the screen, so type the value itself (a name, number, date, or address) into each yellow cell.</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>Data: 8 rows, in the Excel Table 'tblPayers'</t>
+          <t>Data: 8 rows, in the Excel Table 'tblPayers' (hidden: unhide it when a task asks)</t>
         </is>
       </c>
     </row>
@@ -1049,14 +1049,14 @@
     <row r="2" ht="34" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>Every task uses the Patients sheet (500 patients, rows 2–501) unless it says otherwise. No formulas needed: navigate, look, and type what you find. Mac users: for Ctrl+arrow shortcuts such as Ctrl+↓ and Ctrl+Shift+↓, press ⌘ instead of Ctrl.</t>
+          <t>Every task uses the Patients sheet (500 patients, rows 2–501) unless it says otherwise. No formulas needed: navigate, look, and type what you find. Mac users: for Ctrl + arrow shortcuts such as Ctrl + ↓ and Ctrl + Shift + ↓, press ⌘ instead of Ctrl.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Type a formula or value in each yellow cell. The Check column turns green when your answer matches. Stuck? Read the hint, then the lesson guide. Answers: right-click a sheet tab → Unhide… → 'Answer Key'.</t>
+          <t>Type the value you find (a name, number, date, or address) in each yellow cell. The Check column turns green when your answer matches. Stuck? Read the hint, then the lesson guide. Answers: right-click a sheet tab → Unhide… → 'Answer Key'.</t>
         </is>
       </c>
     </row>
@@ -1115,7 +1115,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="51" customHeight="1">
+    <row r="7" ht="66" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>2</t>
@@ -1123,12 +1123,12 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>What is the address of the bottom-right cell of the patient data? From A1, press Ctrl+↓ to find the last row, go back with Ctrl+↑, then press Ctrl+→ to find the last column. Type the address as column letter + row number (like B12).</t>
+          <t>What is the address of the bottom-right cell of the patient data? From A1, press Ctrl + ↓ to find the last row, go back with Ctrl + ↑, then press Ctrl + → to find the last column. Type the address as column letter + row number (like B12).</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>Column letter from Ctrl+→, row number from Ctrl+↓. Ctrl+End confirms</t>
+          <t>Column letter from Ctrl + →, row number from Ctrl + ↓. Ctrl + End confirms</t>
         </is>
       </c>
       <c r="D7" s="20" t="n"/>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Use the Name Box to go to cell A600, which is in an empty row below the data, then press Ctrl+→. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
+          <t>Use the Name Box to go to cell A600, which is in an empty row below the data, then press Ctrl + →. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
         </is>
       </c>
       <c r="C8" s="19" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="B9" s="18" t="inlineStr">
         <is>
-          <t>Click M1 (the PCPProviderID header) and press Ctrl+↓ once. On which row number does Excel stop?</t>
+          <t>Click M1 (the PCPProviderID header) and press Ctrl + ↓ once. On which row number does Excel stop?</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Ctrl+arrow stops at the edge of a block of filled cells</t>
+          <t>Ctrl + arrow stops at the edge of a block of filled cells</t>
         </is>
       </c>
       <c r="D9" s="22" t="n"/>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Select the WeightLb values O2:O501 with Go To: press F5 or Ctrl+G (Mac: Control+G), type O2:O501, and press Enter. What is the average weight in pounds? Round to 1 decimal place.</t>
+          <t>Select the WeightLb values O2:O501 with Go To: press F5 or Ctrl + G (Mac: Control + G), type O2:O501, and press Enter. What is the average weight in pounds? Round to 1 decimal place.</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl+Shift+↓ to select every date of birth. What is the date of birth of the oldest patient? Type it as month/day/year, the way the status bar shows it. (If your computer uses day/month dates, type the month as a word instead, such as 15 Mar 1950.)</t>
+          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl + Shift + ↓ to select every date of birth. What is the date of birth of the oldest patient? Type it as month/day/year, the way the status bar shows it. (If your computer uses day/month dates, type the month as a word instead, such as 15 Mar 1950.)</t>
         </is>
       </c>
       <c r="C12" s="19" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>How many patients live in Millbrook? On the Patients sheet, click a single cell such as A1 so Find searches the whole sheet. Then press Ctrl+F (Mac: Control+F), type Millbrook, click Find All, and read the count at the bottom of the dialog.</t>
+          <t>How many patients live in Millbrook? On the Patients sheet, click a single cell such as A1 so Find searches the whole sheet. Then press Ctrl + F (Mac: Control + F), type Millbrook, click Find All, and read the count at the bottom of the dialog.</t>
         </is>
       </c>
       <c r="C13" s="19" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl+F (Mac: Control+F) to find patient PT12376. What is that patient's phone number?</t>
+          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl + F (Mac: Control + F) to find patient PT12376. What is that patient's phone number?</t>
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr">
@@ -38971,14 +38971,14 @@
     <row r="2" ht="64" customHeight="1">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>The population-health team is starting a blood-pressure outreach program and will build its mailing list from this patient index. Before the letters go out, the data steward asks you to check four facts. Set up the Patients sheet first: if you froze panes earlier, choose View → Freeze Panes → Unfreeze Panes. Then press Ctrl+Home (Mac: Control+Home), click B2, and choose View → Freeze Panes → Freeze Panes so the headers and the PatientID column stay in view. Also turn on Minimum and Maximum in the status bar. You'll look everything up on the Patients sheet and type your answers on the Bonus sheet, without a single formula.</t>
+          <t>The population-health team is starting a blood-pressure outreach program and will build its mailing list from this patient index. Before the letters go out, the data steward asks you to check four facts. Set up the Patients sheet first: if you froze panes earlier, choose View → Freeze Panes → Unfreeze Panes. Then press Ctrl + Home (Mac: Control + Home), click B2, and choose View → Freeze Panes → Freeze Panes so the headers and the PatientID column stay in view. Also turn on Minimum and Maximum in the status bar. You'll look everything up on the Patients sheet and type your answers on the Bonus sheet, without a single formula.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Type a formula or value in each yellow cell. The Check column turns green when your answer matches. Stuck? Read the hint, then the lesson guide. Answers: right-click a sheet tab → Unhide… → 'Bonus Key'.</t>
+          <t>Type the value you find in each yellow cell. The Check column turns green when your answer matches. Stuck? Read the hint, then the lesson guide. Answers: right-click a sheet tab → Unhide… → 'Bonus Key'.</t>
         </is>
       </c>
     </row>
@@ -39023,7 +39023,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>Each outreach letter is signed by the patient's primary care provider (PCP), and a blank PCPProviderID means no PCP is on file. Use Go To (F5 or Ctrl+G, Mac: Control+G) to select M2:M501. How many of the 500 patients have no PCP?</t>
+          <t>Each outreach letter is signed by the patient's primary care provider (PCP), and a blank PCPProviderID means no PCP is on file. Use Go To (F5 or Ctrl + G, Mac: Control + G) to select M2:M501. How many of the 500 patients have no PCP?</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
@@ -39045,7 +39045,7 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>The program targets every patient with hypertension, coded HTN. Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl+F (Mac: Control+F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN. How many patients have HTN anywhere in their ChronicConditions list?</t>
+          <t>The program targets every patient with hypertension, coded HTN. Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl + F (Mac: Control + F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN. How many patients have HTN anywhere in their ChronicConditions list?</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
@@ -39094,7 +39094,7 @@
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>Status bar Maximum, then Ctrl+F for that number</t>
+          <t>Status bar Maximum, then Ctrl + F for that number</t>
         </is>
       </c>
       <c r="D9" s="20" t="n"/>
@@ -39226,7 +39226,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>What is the address of the bottom-right cell of the patient data? From A1, press Ctrl+↓ to find the last row, go back with Ctrl+↑, then press Ctrl+→ to find the last column. Type the address as column letter + row number (like B12).</t>
+          <t>What is the address of the bottom-right cell of the patient data? From A1, press Ctrl + ↓ to find the last row, go back with Ctrl + ↑, then press Ctrl + → to find the last column. Type the address as column letter + row number (like B12).</t>
         </is>
       </c>
       <c r="C6" s="30" t="inlineStr">
@@ -39236,9 +39236,9 @@
       </c>
       <c r="D6" s="31" t="inlineStr">
         <is>
-          <t>1. Click A1 and press Ctrl+↓: the active cell becomes A501.
-2. Press Ctrl+↑ to return to A1, then Ctrl+→: the active cell becomes Q1.
-3. Combine them: Q501. Press Ctrl+End (Mac: Control+End, or Control+Fn+→) to confirm. It jumps straight there.</t>
+          <t>1. Click A1 and press Ctrl + ↓: the active cell becomes A501.
+2. Press Ctrl + ↑ to return to A1, then Ctrl + →: the active cell becomes Q1.
+3. Combine them: Q501. Press Ctrl + End (Mac: Control + End, or Control + Fn + →) to confirm. It jumps straight there.</t>
         </is>
       </c>
       <c r="E6" cm="1" s="18">
@@ -39247,11 +39247,11 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Ctrl+arrow jumps to the edge of the block of filled cells. Column A and row 1 have no gaps, so the jumps land on the true last row (501: 500 patients plus the header row) and the true last column (Q). Ctrl+End goes straight to the last used cell, Q501. The hidden column I doesn't change the answer, because hiding a column doesn't remove it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="66" customHeight="1">
+          <t>Ctrl + arrow jumps to the edge of the block of filled cells. Column A and row 1 have no gaps, so the jumps land on the true last row (501: 500 patients plus the header row) and the true last column (Q). Ctrl + End goes straight to the last used cell, Q501. The hidden column I doesn't change the answer, because hiding a column doesn't remove it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="81" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
           <t>3</t>
@@ -39259,7 +39259,7 @@
       </c>
       <c r="B7" s="18" t="inlineStr">
         <is>
-          <t>Use the Name Box to go to cell A600, which is in an empty row below the data, then press Ctrl+→. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
+          <t>Use the Name Box to go to cell A600, which is in an empty row below the data, then press Ctrl + →. Excel races across the empty row to the very last column of the worksheet. What is the address of the cell you land on?</t>
         </is>
       </c>
       <c r="C7" s="30" t="inlineStr">
@@ -39270,8 +39270,8 @@
       <c r="D7" s="31" t="inlineStr">
         <is>
           <t>1. Type A600 in the Name Box and press Enter.
-2. Press Ctrl+→. The Name Box shows XFD600.
-3. Press Ctrl+← to come back to column A.</t>
+2. Press Ctrl + →. The Name Box shows XFD600.
+3. Press Ctrl + ← to come back to column A.</t>
         </is>
       </c>
       <c r="E7" cm="1" s="18">
@@ -39280,11 +39280,11 @@
       </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
-          <t>When the row is empty, Ctrl+→ has no data to stop at, so it goes to the edge of the sheet: column XFD, the 16,384th column. Ctrl+↓ in an empty column goes to row 1,048,576. Every modern worksheet has exactly 1,048,576 rows × 16,384 columns.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="81" customHeight="1">
+          <t>When the row is empty, Ctrl + → has no data to stop at, so it goes to the edge of the sheet: column XFD, the 16,384th column. Ctrl + ↓ in an empty column goes to row 1,048,576. Every modern worksheet has exactly 1,048,576 rows × 16,384 columns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="96" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
           <t>4</t>
@@ -39292,7 +39292,7 @@
       </c>
       <c r="B8" s="18" t="inlineStr">
         <is>
-          <t>Click M1 (the PCPProviderID header) and press Ctrl+↓ once. On which row number does Excel stop?</t>
+          <t>Click M1 (the PCPProviderID header) and press Ctrl + ↓ once. On which row number does Excel stop?</t>
         </is>
       </c>
       <c r="C8" s="30" t="n">
@@ -39301,7 +39301,7 @@
       <c r="D8" s="31" t="inlineStr">
         <is>
           <t>1. Click M1 (or type M1 in the Name Box).
-2. Press Ctrl+↓. The Name Box shows M34.</t>
+2. Press Ctrl + ↓. The Name Box shows M34.</t>
         </is>
       </c>
       <c r="E8" cm="1" s="18">
@@ -39310,7 +39310,7 @@
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>M35 is empty because that patient has no primary care provider on file. Ctrl+↓ stops at the last filled cell before the gap, M34, even though the data continues to row 501. Never assume Ctrl+↓ found the bottom of a column with blanks. Check the row number, or press Ctrl+↓ again to keep jumping.</t>
+          <t>M35 is empty because that patient has no primary care provider on file. Ctrl + ↓ stops at the last filled cell before the gap, M34, even though the data continues to row 501. Never assume Ctrl + ↓ found the bottom of a column with blanks. Check the row number, or press Ctrl + ↓ again to keep jumping.</t>
         </is>
       </c>
     </row>
@@ -39340,7 +39340,7 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>The status bar's Count counts every non-empty cell, text included, so it counts the email addresses and skips the blanks. Typing the range in the Name Box selects exactly 500 cells. Ctrl+Shift+↓ from J2 would be a trap, because the Email column has gaps: it would select only J2:J3. In a Table you can also click any Email cell and press Ctrl+Space (Mac: Control+Space) to select just that column's data.</t>
+          <t>The status bar's Count counts every non-empty cell, text included, so it counts the email addresses and skips the blanks. Typing the range in the Name Box selects exactly 500 cells. Ctrl + Shift + ↓ from J2 would be a trap, because the Email column has gaps: it would select only J2:J3. In a Table you can also click any Email cell and press Ctrl + Space (Mac: Control + Space) to select just that column's data.</t>
         </is>
       </c>
     </row>
@@ -39352,7 +39352,7 @@
       </c>
       <c r="B10" s="18" t="inlineStr">
         <is>
-          <t>Select the WeightLb values O2:O501 with Go To: press F5 or Ctrl+G (Mac: Control+G), type O2:O501, and press Enter. What is the average weight in pounds? Round to 1 decimal place.</t>
+          <t>Select the WeightLb values O2:O501 with Go To: press F5 or Ctrl + G (Mac: Control + G), type O2:O501, and press Enter. What is the average weight in pounds? Round to 1 decimal place.</t>
         </is>
       </c>
       <c r="C10" s="32" t="n">
@@ -39360,7 +39360,7 @@
       </c>
       <c r="D10" s="31" t="inlineStr">
         <is>
-          <t>1. Press F5 (or Ctrl+G), type O2:O501 in Reference, press Enter.
+          <t>1. Press F5 (or Ctrl + G), type O2:O501 in Reference, press Enter.
 2. Read Average on the status bar and round it to 1 decimal place.</t>
         </is>
       </c>
@@ -39382,7 +39382,7 @@
       </c>
       <c r="B11" s="18" t="inlineStr">
         <is>
-          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl+Shift+↓ to select every date of birth. What is the date of birth of the oldest patient? Type it as month/day/year, the way the status bar shows it. (If your computer uses day/month dates, type the month as a word instead, such as 15 Mar 1950.)</t>
+          <t>Turn on Minimum in the status bar: right-click the status bar and tick Minimum. Then click cell F2 (the first DOB) and press Ctrl + Shift + ↓ to select every date of birth. What is the date of birth of the oldest patient? Type it as month/day/year, the way the status bar shows it. (If your computer uses day/month dates, type the month as a word instead, such as 15 Mar 1950.)</t>
         </is>
       </c>
       <c r="C11" s="34" t="n">
@@ -39391,7 +39391,7 @@
       <c r="D11" s="31" t="inlineStr">
         <is>
           <t>1. Right-click the status bar and tick Minimum (and Maximum while you're there).
-2. Click cell F2 and press Ctrl+Shift+↓ to select F2:F501.
+2. Click cell F2 and press Ctrl + Shift + ↓ to select F2:F501.
 3. Read Minimum on the status bar.</t>
         </is>
       </c>
@@ -39401,7 +39401,7 @@
       </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
-          <t>Excel stores dates as numbers that grow by 1 each day, so the earliest date is the smallest number and Minimum finds it. The status bar shows it as a date because the cells are formatted as dates. (If you see a plain number such as 9534 instead, that's the date's serial number, and the check accepts it.) Ctrl+Shift+↓ is safe here because the DOB column has no blanks.</t>
+          <t>Excel stores dates as numbers that grow by 1 each day, so the earliest date is the smallest number and Minimum finds it. The status bar shows it as a date because the cells are formatted as dates. (If you see a plain number such as 9534 instead, that's the date's serial number, and the check accepts it.) Ctrl + Shift + ↓ is safe here because the DOB column has no blanks.</t>
         </is>
       </c>
     </row>
@@ -39413,7 +39413,7 @@
       </c>
       <c r="B12" s="18" t="inlineStr">
         <is>
-          <t>How many patients live in Millbrook? On the Patients sheet, click a single cell such as A1 so Find searches the whole sheet. Then press Ctrl+F (Mac: Control+F), type Millbrook, click Find All, and read the count at the bottom of the dialog.</t>
+          <t>How many patients live in Millbrook? On the Patients sheet, click a single cell such as A1 so Find searches the whole sheet. Then press Ctrl + F (Mac: Control + F), type Millbrook, click Find All, and read the count at the bottom of the dialog.</t>
         </is>
       </c>
       <c r="C12" s="30" t="n">
@@ -39422,7 +39422,7 @@
       <c r="D12" s="31" t="inlineStr">
         <is>
           <t>1. Click A1 (one cell, so Find searches the whole sheet).
-2. Press Ctrl+F, type Millbrook, and click Find All.
+2. Press Ctrl + F, type Millbrook, and click Find All.
 3. Read '… cell(s) found' at the bottom of the dialog.</t>
         </is>
       </c>
@@ -39444,7 +39444,7 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl+F (Mac: Control+F) to find patient PT12376. What is that patient's phone number?</t>
+          <t>Column I is hidden (the column letters jump from H to J). Unhide it, then click cell A1 and use Ctrl + F (Mac: Control + F) to find patient PT12376. What is that patient's phone number?</t>
         </is>
       </c>
       <c r="C13" s="30" t="inlineStr">
@@ -39454,8 +39454,8 @@
       </c>
       <c r="D13" s="31" t="inlineStr">
         <is>
-          <t>1. Click the H column header, Shift+click the J header, then right-click → Unhide.
-2. Click A1, press Ctrl+F, type PT12376, click Find Next, then close the dialog.
+          <t>1. Click the H column header, Shift + click the J header, then right-click → Unhide.
+2. Click A1, press Ctrl + F, type PT12376, click Find Next, then close the dialog.
 3. Read column I on row 298.</t>
         </is>
       </c>
@@ -39487,8 +39487,8 @@
       </c>
       <c r="D14" s="31" t="inlineStr">
         <is>
-          <t>1. On the Patients sheet, click A1, press Ctrl+F, and find PT13312: row 415, payer ID PY06.
-2. Right-click any sheet tab → Unhide… → Payers → OK.
+          <t>1. On the Patients sheet, click A1, press Ctrl + F, and find PT13312: row 415, payer ID PY06.
+2. Right-click any sheet tab → Unhide…, pick Payers, and click OK.
 3. On the Payers sheet, PY06 is Summit Choice PPO.</t>
         </is>
       </c>
@@ -39552,7 +39552,7 @@
       <c r="D16" s="31" t="inlineStr">
         <is>
           <t>1. Click C2.
-2. View → Freeze Panes → Freeze Panes.
+2. Choose View → Freeze Panes → Freeze Panes.
 3. Scroll down and right: row 1 and columns A:B stay put. (View → Freeze Panes → Unfreeze Panes undoes it.)</t>
         </is>
       </c>
@@ -39648,7 +39648,7 @@
       </c>
       <c r="B5" s="18" t="inlineStr">
         <is>
-          <t>Each outreach letter is signed by the patient's primary care provider (PCP), and a blank PCPProviderID means no PCP is on file. Use Go To (F5 or Ctrl+G, Mac: Control+G) to select M2:M501. How many of the 500 patients have no PCP?</t>
+          <t>Each outreach letter is signed by the patient's primary care provider (PCP), and a blank PCPProviderID means no PCP is on file. Use Go To (F5 or Ctrl + G, Mac: Control + G) to select M2:M501. How many of the 500 patients have no PCP?</t>
         </is>
       </c>
       <c r="C5" s="30" t="n">
@@ -39679,7 +39679,7 @@
       </c>
       <c r="B6" s="18" t="inlineStr">
         <is>
-          <t>The program targets every patient with hypertension, coded HTN. Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl+F (Mac: Control+F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN. How many patients have HTN anywhere in their ChronicConditions list?</t>
+          <t>The program targets every patient with hypertension, coded HTN. Click a single cell such as A1, so Find searches the whole sheet rather than the column you just selected. Press Ctrl + F (Mac: Control + F), click Options &gt;&gt; and make sure Match entire cell contents is OFF, then Find All for HTN. How many patients have HTN anywhere in their ChronicConditions list?</t>
         </is>
       </c>
       <c r="C6" s="30" t="n">
@@ -39687,7 +39687,7 @@
       </c>
       <c r="D6" s="31" t="inlineStr">
         <is>
-          <t>1. Click A1, then Ctrl+F → Options &gt;&gt; → untick Match entire cell contents.
+          <t>1. Click A1, press Ctrl + F, click Options &gt;&gt;, and untick Match entire cell contents.
 2. Type HTN and click Find All.
 3. Read the count at the bottom of the dialog.</t>
         </is>
@@ -39752,7 +39752,7 @@
       <c r="D8" s="31" t="inlineStr">
         <is>
           <t>1. Select O2:O501 (Name Box or Go To) and read Maximum: 319.2.
-2. With the weights still selected, press Ctrl+F → Find what: 319.2 → Find Next. (Match entire cell contents can be on or off here, because no other cell on the sheet contains 319.2.)
+2. With the weights still selected, press Ctrl + F, type 319.2 in Find what, and click Find Next. (Match entire cell contents can be on or off here, because no other cell on the sheet contains 319.2.)
 3. Excel selects O474. The frozen column A shows PT13784.</t>
         </is>
       </c>

</xml_diff>